<commit_message>
Fix Type column display inversion and rename FB columns in comparison xlsx
- Fix NC/NO display inversion in comparison Type column (exp_no=True → NO, False → NC)
- Rename comparison headers FBOPN→FBOPN_EN, FBCLS→FBCLS_EN for Exp and DB columns
- Fix stale docstring comments in run.py (NC→False, NO→True)
- Regenerated all 5 comparison xlsx and updated db files

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Brew_Comparison.xlsx
+++ b/Brew_Comparison.xlsx
@@ -78,11 +78,11 @@
   </si>
   <si>
     <t>Exp
-FBOPN</t>
+FBOPN_EN</t>
   </si>
   <si>
     <t>Exp
-FBCLS</t>
+FBCLS_EN</t>
   </si>
   <si>
     <t>DB
@@ -102,11 +102,11 @@
   </si>
   <si>
     <t>DB
-FBOPN</t>
+FBOPN_EN</t>
   </si>
   <si>
     <t>DB
-FBCLS</t>
+FBCLS_EN</t>
   </si>
   <si>
     <t>Match</t>
@@ -130,7 +130,7 @@
     <t>X</t>
   </si>
   <si>
-    <t>NO</t>
+    <t>NC</t>
   </si>
   <si>
     <t>T</t>
@@ -172,7 +172,7 @@
     <t>EM - 212</t>
   </si>
   <si>
-    <t>NC</t>
+    <t>NO</t>
   </si>
   <si>
     <t>AV220-1</t>

</xml_diff>